<commit_message>
Vacante comercial: version final en el archivo oficial, eliminado el auxiliar v2
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/recursos/comercial/INDUCCION_COMERCIAL/contratacion comercial/POST_LINKEDIN_VACANTE.xlsx
+++ b/recursos/comercial/INDUCCION_COMERCIAL/contratacion comercial/POST_LINKEDIN_VACANTE.xlsx
@@ -10,6 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="POST LINKEDIN" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PIEZA GRAFICA" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PARA BRIAN" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PORTALES (ACADEMIA)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MENSAJE DIRECTO" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -568,7 +570,7 @@
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>Envía tu hoja de vida a [CORREO DE RECEPCIÓN] con el asunto "Comercial Heiiu" y, esto es lo importante, un audio o video de 1 minuto contándonos la venta más difícil que has cerrado y cómo la lograste. Sin el audio no revisamos la hoja de vida.</t>
+          <t>Envía tu hoja de vida a auxiliaradministrativo@heiiu.com con el asunto "Comercial Heiiu" y, esto es lo importante, un audio o video de 1 minuto contándonos la venta más difícil que has cerrado y cómo la lograste. Sin el audio no revisamos la hoja de vida.</t>
         </is>
       </c>
     </row>
@@ -701,7 +703,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>INSTRUCCIONES DE PUBLICACIÓN</t>
+          <t>PARA BRIAN — SOLO LINKEDIN Y REDES</t>
         </is>
       </c>
     </row>
@@ -711,42 +713,202 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>1. Se publica desde la página de empresa de Heiiu en LinkedIn, y Diana lo comparte desde su perfil personal el mismo día: el perfil personal tiene más alcance orgánico que la página.</t>
+          <t>1. PIEZA PRINCIPAL: crear la vacante gratuita en LinkedIn Empleos desde la página de empresa de Heiiu, con el texto del post (título: Ejecutivo(a) Comercial de Planta · ubicación: Bucaramanga · presencial · tiempo completo). Aparece por búsqueda, no depende de seguidores.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>2. Además, crear la vacante gratuita en LinkedIn Empleos con el mismo texto (título: Ejecutivo(a) Comercial de Planta · ubicación: Bucaramanga · presencial · tiempo completo).</t>
+          <t>2. Publicar el post en la página de Heiiu con la pieza gráfica, y compartirlo desde su perfil como apoyo, siempre enlazando a la vacante oficial de Heiiu.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>3. Si se le pone pauta: segmentar Bucaramanga y área metropolitana, cargos actuales tipo asesor comercial, ejecutivo de ventas o ejecutivo de cuenta, sectores seguros, educación, telecomunicaciones, servicios financieros y planes de salud o exequiales.</t>
+          <t>3. Replicar la pieza gráfica en Instagram y Facebook de la academia.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>4. Replicar el texto de la pieza gráfica en Instagram y Facebook de la academia, y en los portales de empleo gratuitos (Computrabajo, elempleo, Magneto).</t>
+          <t>4. Si se le pone pauta: segmentar Bucaramanga y área metropolitana, cargos actuales tipo asesor comercial, ejecutivo de ventas o ejecutivo de cuenta, sectores seguros, educación, telecomunicaciones, servicios financieros y planes de salud o exequiales.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>5. Antes de publicar: reemplazar [CORREO DE RECEPCIÓN] por el correo donde van a llegar las hojas de vida.</t>
+          <t>5. Las hojas de vida llegan a auxiliaradministrativo@heiiu.com con el asunto "Comercial Heiiu".</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="120" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PORTALES DE EMPLEO GRATUITOS — LOS PUBLICA LA ACADEMIA, NO BRIAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Dónde: Computrabajo · Magneto · elempleo · Servicio Público de Empleo (Agencia de Cajasan o Comfenalco) · grupos de empleo de Bucaramanga en Facebook.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Datos para llenar los formularios:</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>· Cargo: Ejecutivo(a) Comercial de Planta</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>· Empresa: Heiiu English Academy (Global Teacher S.A.S.)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>6. El filtro del audio no se negocia: quien no manda audio queda descartado sin revisar. Es la primera prueba del cargo.</t>
+          <t>· Ciudad: Bucaramanga · presencial · tiempo completo</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>· Contrato: término fijo a un año</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>· Salario: $2.000.000 + comisiones + prestaciones de ley</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>· Experiencia: mínimo 2 años en venta de intangibles</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>· Descripción: copiar el texto de la hoja POST LINKEDIN, sin los hashtags.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>· Contacto: auxiliaradministrativo@heiiu.com, asunto "Comercial Heiiu".</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>Filtro al recibir: quien no mande el audio o video de 1 minuto queda descartado sin revisar. A los que sí lo manden se les aplica la guía de entrevista (GUIA_ENTREVISTA_COMERCIAL_v3).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="120" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>MENSAJE DIRECTO PARA VENDEDORES QUE YA ESTÁN TRABAJANDO (búsqueda activa en LinkedIn)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Hola [NOMBRE], vi tu perfil y tu experiencia en ventas en [EMPRESA / SECTOR]. En Heiiu English Academy, en Bucaramanga, estamos buscando UNA persona comercial de planta: contrato laboral a un año, básico de $2.000.000 más comisiones sin techo, y dos aumentos de básico en el primer año atados a resultados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Es un cargo de prospección y cierre, para alguien a quien le guste salir a buscar el negocio. Si te interesa conocer los detalles, o conoces a alguien con ese perfil, cuéntame y te comparto la información completa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>A quién buscar: personas en Bucaramanga con cargos de asesor comercial, ejecutivo de ventas o ejecutivo de cuenta en seguros, planes exequiales o de salud, telecomunicaciones, servicios financieros o educación. Meta: 20 mensajes directos en la primera semana.</t>
         </is>
       </c>
     </row>

</xml_diff>